<commit_message>
Logical And Conditional Functions
</commit_message>
<xml_diff>
--- a/Excel Practice @ Day 03 New.xlsx
+++ b/Excel Practice @ Day 03 New.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35ad282c83c5c77b/Desktop/Codegnan DA-HYD-026/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{71B56813-AC0B-458C-A242-0E8D5DA3824E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59C097AA-0D14-49C1-856E-37DB27E40B1A}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{71B56813-AC0B-458C-A242-0E8D5DA3824E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6310F2F7-1448-41FC-8905-12513BC45A5B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,6 +24,8 @@
     <definedName name="Dept">Patient_Data!$E$2:$E$41</definedName>
     <definedName name="Gender">Patient_Data!$D$2:$D$41</definedName>
     <definedName name="Insurance">Patient_Data!$J$2:$J$41</definedName>
+    <definedName name="noofstays">Patient_Data!$M$2:$M$41</definedName>
+    <definedName name="Payment_status">Patient_Data!$L$2:$L$41</definedName>
     <definedName name="Stay">Patient_Data!$M$2:$M$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -4662,7 +4664,10 @@
         <f>COUNTIF(Gender,D38)</f>
         <v>20</v>
       </c>
-      <c r="K49" s="8"/>
+      <c r="K49" s="8">
+        <f>COUNTIF(Department,E15)</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="50" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E50" t="s">
@@ -4672,6 +4677,10 @@
         <f>AVERAGEIF(Department,E39,Bills)</f>
         <v>25571.428571428572</v>
       </c>
+      <c r="K50" s="8">
+        <f>AVERAGEIF(Department,E18,Bills)</f>
+        <v>25571.428571428572</v>
+      </c>
     </row>
     <row r="51" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E51" t="s">
@@ -4681,6 +4690,10 @@
         <f>SUMIF(J2:J41,J22,Bills)</f>
         <v>499500</v>
       </c>
+      <c r="K51" s="8">
+        <f>SUMIF(Insurance,J3,Bills)</f>
+        <v>499500</v>
+      </c>
     </row>
     <row r="52" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E52" t="s">
@@ -4690,11 +4703,19 @@
         <f>COUNTIF(L2:L41,L25)</f>
         <v>10</v>
       </c>
+      <c r="K52" s="8">
+        <f>COUNTIF(L2:L41,L5)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="53" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E53" t="s">
         <v>126</v>
       </c>
+      <c r="K53" s="8">
+        <f ca="1">SUMIF(L1:L41,L5,Bills)</f>
+        <v>286300</v>
+      </c>
     </row>
     <row r="54" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E54" t="s">
@@ -4704,6 +4725,10 @@
         <f>SUMIFS(Bills,Department,E41,J2:J41,J25)</f>
         <v>275500</v>
       </c>
+      <c r="K54" s="8">
+        <f>SUMIFS(Bills,Department,E5,Insurance,J3)</f>
+        <v>275500</v>
+      </c>
     </row>
     <row r="55" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E55" t="s">
@@ -4713,11 +4738,19 @@
         <f>COUNTIFS(Department,E41,L2:L41,L28)</f>
         <v>4</v>
       </c>
+      <c r="K55" s="8">
+        <f>COUNTIFS(Department,E2,L2:L41,L5)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="56" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E56" t="s">
         <v>129</v>
       </c>
+      <c r="K56" s="8">
+        <f>AVERAGEIF(Insurance,J2,Bills)</f>
+        <v>25766.666666666668</v>
+      </c>
     </row>
     <row r="57" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E57" t="s">
@@ -4727,6 +4760,10 @@
         <f>COUNTIF(Bills,"&gt;40000")</f>
         <v>9</v>
       </c>
+      <c r="K57" s="8">
+        <f>COUNTIF(Bills, "&gt; 40000")</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="58" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E58" t="s">
@@ -4736,11 +4773,19 @@
         <f>SUMIF(Bills,"&gt;40000",Bills)</f>
         <v>508000</v>
       </c>
+      <c r="K58" s="8">
+        <f>SUMIF(Bills,"&gt;40000",Bills)</f>
+        <v>508000</v>
+      </c>
     </row>
     <row r="59" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E59" t="s">
         <v>132</v>
       </c>
+      <c r="K59" s="8">
+        <f>COUNTIF(noofstays,"&gt;5")</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="60" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E60" t="s">
@@ -4750,6 +4795,10 @@
         <f>SUMIF(Stay,"&gt;5",Bills)</f>
         <v>582000</v>
       </c>
+      <c r="K60" s="8">
+        <f>SUMIF(noofstays,"&gt;5",Bills)</f>
+        <v>582000</v>
+      </c>
     </row>
     <row r="61" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E61" t="s">
@@ -4759,11 +4808,19 @@
         <f>SUMIFS(Bills,Department,E41,Stay,"&gt;5")</f>
         <v>320000</v>
       </c>
+      <c r="K61" s="8">
+        <f>SUMIFS(Bills,Department,E2,noofstays,"&gt;5")</f>
+        <v>320000</v>
+      </c>
     </row>
     <row r="62" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E62" t="s">
         <v>135</v>
       </c>
+      <c r="K62" s="8">
+        <f>AVERAGEIF(L2:L41,L5,noofstays)</f>
+        <v>5.8</v>
+      </c>
     </row>
     <row r="63" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E63" t="s">
@@ -4773,20 +4830,36 @@
         <f>_xlfn.MAXIFS(Bills,Department,E41)</f>
         <v>76000</v>
       </c>
+      <c r="K63" s="8">
+        <f>_xlfn.MAXIFS(Bills,Department,E2)</f>
+        <v>76000</v>
+      </c>
     </row>
     <row r="64" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E64" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="65" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="K64" s="8">
+        <f>_xlfn.MINIFS(Bills,Department,E3)</f>
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="65" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E65" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="66" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="K65" s="8">
+        <f>COUNTIFS(Department,E2,L2:L41,L5)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E66" t="s">
         <v>142</v>
+      </c>
+      <c r="K66" s="8">
+        <f>AVERAGEIFS(Bills,Department,E2,Insurance,J3)</f>
+        <v>55100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>